<commit_message>
feat: skrining remaja done
</commit_message>
<xml_diff>
--- a/dataset/dewasa.xlsx
+++ b/dataset/dewasa.xlsx
@@ -2605,10 +2605,7 @@
       </c>
       <c r="FU2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAILED: Locator.click: Target page, context or browser has been closed
-Call log:
-  - waiting for locator("div.cursor-pointer.px-3").filter(has_text="Sedang Pemeriksaan")
-</t>
+          <t>FAILED: Pasien tidak ditemukan pada semua status pemeriksaan.</t>
         </is>
       </c>
     </row>
@@ -3444,7 +3441,7 @@
       </c>
       <c r="FU3" t="inlineStr">
         <is>
-          <t>FAILED: Page.goto: Target page, context or browser has been closed</t>
+          <t>SUCCESS</t>
         </is>
       </c>
     </row>
@@ -3587,7 +3584,7 @@
       <c r="FT4" s="2" t="n"/>
       <c r="FU4" t="inlineStr">
         <is>
-          <t>FAILED: Page.goto: Target page, context or browser has been closed</t>
+          <t>FAILED: Pasien tidak ditemukan pada semua status pemeriksaan.</t>
         </is>
       </c>
     </row>

</xml_diff>